<commit_message>
feat: insights ingestão, de-para, purge e stack admin
- Insights: hooks e painel com dados reais; admin de-para produtos e exclusão cliente
  com RPC (cascade + reconciliação total_nfs/total_itens); scripts import/enrich/delete.
- Migrations SQL 008–017 em docs/migrations (perfil, analytics, clientes, purge, totais).
- Distribuidor: de-para produtos no admin, scripts faturamento/normalização; templates.
- Excelência e integrações documentais (SUPABASE_PROJECT, CHECKLIST, AGENTS).
- .gitignore: extracto GA_VGF faturamento bruto (≥100 MB GitHub) fora do repositório.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/templates/template_relatorio_vendas.xlsx
+++ b/docs/templates/template_relatorio_vendas.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P4"/>
+  <dimension ref="A1:Q4"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -415,6 +415,7 @@
     <col min="14" max="14" width="18.83203125" customWidth="1"/>
     <col min="15" max="15" width="18.83203125" customWidth="1"/>
     <col min="16" max="16" width="18.83203125" customWidth="1"/>
+    <col min="17" max="17" width="18.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -428,42 +429,45 @@
         <v>cnpj_cliente</v>
       </c>
       <c r="D1" t="str">
+        <v>razao_social</v>
+      </c>
+      <c r="E1" t="str">
         <v>nome_cliente</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>codigo_vendedor</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>nome_vendedor</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>codigo_supervisor</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>nome_supervisor</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>codigo_gerente</v>
       </c>
-      <c r="J1" t="str">
+      <c r="K1" t="str">
         <v>nome_gerente</v>
       </c>
-      <c r="K1" t="str">
+      <c r="L1" t="str">
         <v>sku</v>
       </c>
-      <c r="L1" t="str">
+      <c r="M1" t="str">
         <v>descricao_produto</v>
       </c>
-      <c r="M1" t="str">
+      <c r="N1" t="str">
         <v>quantidade</v>
       </c>
-      <c r="N1" t="str">
+      <c r="O1" t="str">
         <v>unidade</v>
       </c>
-      <c r="O1" t="str">
+      <c r="P1" t="str">
         <v>valor_unitario</v>
       </c>
-      <c r="P1" t="str">
+      <c r="Q1" t="str">
         <v>valor_total</v>
       </c>
     </row>
@@ -478,42 +482,45 @@
         <v>12345678000199</v>
       </c>
       <c r="D2" t="str">
+        <v>Mercado Exemplo LTDA</v>
+      </c>
+      <c r="E2" t="str">
         <v>Mercado Exemplo</v>
       </c>
-      <c r="E2" t="str">
+      <c r="F2" t="str">
         <v>V001</v>
       </c>
-      <c r="F2" t="str">
+      <c r="G2" t="str">
         <v>João Silva</v>
       </c>
-      <c r="G2" t="str">
+      <c r="H2" t="str">
         <v>S001</v>
       </c>
-      <c r="H2" t="str">
+      <c r="I2" t="str">
         <v>Pedro Costa</v>
       </c>
-      <c r="I2" t="str">
+      <c r="J2" t="str">
         <v>G001</v>
       </c>
-      <c r="J2" t="str">
+      <c r="K2" t="str">
         <v>Maria Gerência</v>
       </c>
-      <c r="K2" t="str">
+      <c r="L2" t="str">
         <v>CAMP-001</v>
       </c>
-      <c r="L2" t="str">
+      <c r="M2" t="str">
         <v>Produto Campestre 1kg</v>
       </c>
-      <c r="M2">
+      <c r="N2">
         <v>10</v>
       </c>
-      <c r="N2" t="str">
+      <c r="O2" t="str">
         <v>UN</v>
       </c>
-      <c r="O2">
+      <c r="P2">
         <v>25.9</v>
       </c>
-      <c r="P2">
+      <c r="Q2">
         <v>259</v>
       </c>
     </row>
@@ -528,42 +535,45 @@
         <v>12345678000199</v>
       </c>
       <c r="D3" t="str">
+        <v>Mercado Exemplo LTDA</v>
+      </c>
+      <c r="E3" t="str">
         <v>Mercado Exemplo</v>
       </c>
-      <c r="E3" t="str">
+      <c r="F3" t="str">
         <v>V001</v>
       </c>
-      <c r="F3" t="str">
+      <c r="G3" t="str">
         <v>João Silva</v>
       </c>
-      <c r="G3" t="str">
+      <c r="H3" t="str">
         <v>S001</v>
       </c>
-      <c r="H3" t="str">
+      <c r="I3" t="str">
         <v>Pedro Costa</v>
       </c>
-      <c r="I3" t="str">
+      <c r="J3" t="str">
         <v>G001</v>
       </c>
-      <c r="J3" t="str">
+      <c r="K3" t="str">
         <v>Maria Gerência</v>
       </c>
-      <c r="K3" t="str">
+      <c r="L3" t="str">
         <v>CAMP-002</v>
       </c>
-      <c r="L3" t="str">
+      <c r="M3" t="str">
         <v>Produto Campestre 500g</v>
       </c>
-      <c r="M3">
+      <c r="N3">
         <v>5</v>
       </c>
-      <c r="N3" t="str">
+      <c r="O3" t="str">
         <v>UN</v>
       </c>
-      <c r="O3">
+      <c r="P3">
         <v>14.5</v>
       </c>
-      <c r="P3">
+      <c r="Q3">
         <v>72.5</v>
       </c>
     </row>
@@ -578,48 +588,51 @@
         <v>98765432000188</v>
       </c>
       <c r="D4" t="str">
+        <v>Supermercado Teste SA</v>
+      </c>
+      <c r="E4" t="str">
         <v>Supermercado Teste</v>
       </c>
-      <c r="E4" t="str">
+      <c r="F4" t="str">
         <v>V001</v>
       </c>
-      <c r="F4" t="str">
+      <c r="G4" t="str">
         <v>João Silva</v>
       </c>
-      <c r="G4" t="str">
+      <c r="H4" t="str">
         <v>S001</v>
       </c>
-      <c r="H4" t="str">
+      <c r="I4" t="str">
         <v>Pedro Costa</v>
       </c>
-      <c r="I4" t="str">
+      <c r="J4" t="str">
         <v>G001</v>
       </c>
-      <c r="J4" t="str">
+      <c r="K4" t="str">
         <v>Maria Gerência</v>
       </c>
-      <c r="K4" t="str">
+      <c r="L4" t="str">
         <v>CAMP-001</v>
       </c>
-      <c r="L4" t="str">
+      <c r="M4" t="str">
         <v>Produto Campestre 1kg</v>
       </c>
-      <c r="M4">
+      <c r="N4">
         <v>2</v>
       </c>
-      <c r="N4" t="str">
+      <c r="O4" t="str">
         <v>CX</v>
       </c>
-      <c r="O4">
+      <c r="P4">
         <v>25.9</v>
       </c>
-      <c r="P4">
+      <c r="Q4">
         <v>51.8</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>